<commit_message>
pilot annotation analysis and taxonomy health review
</commit_message>
<xml_diff>
--- a/golden/b01_pilot_labelled.csv.xlsx
+++ b/golden/b01_pilot_labelled.csv.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\hiver-support-agent\golden\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{860DEBFC-111F-450B-A617-EA6840997C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{4FD12EFF-24D3-4D32-9693-CE9A76AC536B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B94DA4A0-C9DE-441E-A2E1-A7DFDBCAE248}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{B94DA4A0-C9DE-441E-A2E1-A7DFDBCAE248}"/>
   </bookViews>
   <sheets>
     <sheet name="b01_pilot_blank" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="558">
   <si>
     <t>annotation_id</t>
   </si>
@@ -652,9 +652,6 @@
     <t>conv_2373654</t>
   </si>
   <si>
-    <t>@AmericanAir The largest plane I’ve ever flown in is the AA 757 and the A321, I’m eager to experience flying on a larger plane.</t>
-  </si>
-  <si>
     <t>b01_0067</t>
   </si>
   <si>
@@ -1394,13 +1391,316 @@
   </si>
   <si>
     <t>Wonderful Flagship Lounge at JFK @AmericanAir https://t.co/6Gmh9xZxpg</t>
+  </si>
+  <si>
+    <t>praise_and_compliment</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>flight_delay</t>
+  </si>
+  <si>
+    <t>OTHER</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Airport shuttle/ground transportation issue; no existing taxonomy category clearly fits.</t>
+  </si>
+  <si>
+    <t>booking_fees_and_fare_rules</t>
+  </si>
+  <si>
+    <t>Cancellation context, but the request is about changing/reusing ticket value.</t>
+  </si>
+  <si>
+    <t>baggage</t>
+  </si>
+  <si>
+    <t>Contains separate delay and lost-baggage issues; also mentions a charge.</t>
+  </si>
+  <si>
+    <t>general_dissatisfaction</t>
+  </si>
+  <si>
+    <t>No specific actionable airline issue is stated</t>
+  </si>
+  <si>
+    <t>Contains a significant flight delay and a separate baggage issue; also mentions a charge from another company.</t>
+  </si>
+  <si>
+    <t>Praises a staff member; flight issue is mentioned but not specific enough to confidently assign a separate operational intent.</t>
+  </si>
+  <si>
+    <t>staff_and_service_complaint</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>Refund/ticket ownership situation; unclear whether this fits booking/fare rules cleanly.</t>
+  </si>
+  <si>
+    <t>Complains about overflow/waiting but the specific underlying support issue is unclear.</t>
+  </si>
+  <si>
+    <t>booking_fee_and_fare_rules</t>
+  </si>
+  <si>
+    <t>Primary issue is an 8-hour delay; compensation request creates a second fare/refund-related aspect.</t>
+  </si>
+  <si>
+    <t>seating_and_upgrade</t>
+  </si>
+  <si>
+    <t>UNCLEAR</t>
+  </si>
+  <si>
+    <t>Only states location/Admirals Club; no clear customer request.</t>
+  </si>
+  <si>
+    <t>boarding_and_gate</t>
+  </si>
+  <si>
+    <t>Delay and gate/ground-crew issue both present; missed connection risk.</t>
+  </si>
+  <si>
+    <t>Spanish; unable to determine intent confidently.</t>
+  </si>
+  <si>
+    <t>No actionable issue stated.</t>
+  </si>
+  <si>
+    <t>loyalty_and_lounge</t>
+  </si>
+  <si>
+    <t>flight_cancellation_rebooking</t>
+  </si>
+  <si>
+    <t>Cancellation plus a separate issue with receiving account credit.</t>
+  </si>
+  <si>
+    <t>No actionable request or specific issue</t>
+  </si>
+  <si>
+    <t>Specific issue does not clearly fit an existing intent; possible customer-service/role issue</t>
+  </si>
+  <si>
+    <t>One-hour delay caused by ground-crew/tow-bar issue; staff criticism is the stated cause rather than a separate issue.</t>
+  </si>
+  <si>
+    <t>Message describes both recurring delays and cancellations; delay is chosen as primary</t>
+  </si>
+  <si>
+    <t>Mentions 500-mile upgrades/benefits, but the exact underlying issue is unclear.</t>
+  </si>
+  <si>
+    <t>refund request</t>
+  </si>
+  <si>
+    <t>Late arrival caused a missed connection; underlying cause of lateness is not explicitly stated</t>
+  </si>
+  <si>
+    <t>I can't understand the message properly</t>
+  </si>
+  <si>
+    <t>Delay explicitly stated; staff member is mentioned as the cause, not a separate request</t>
+  </si>
+  <si>
+    <t>No specific actionable issue is stated.</t>
+  </si>
+  <si>
+    <t>Complaint about paid seat selection and how the seat is represented; fee/fare boundary.</t>
+  </si>
+  <si>
+    <t>Priority/first-class check-in issue does not fit perfectly; paid service and check-in both involved.</t>
+  </si>
+  <si>
+    <t>Positive service-related statement but unusual wording; no support request.</t>
+  </si>
+  <si>
+    <t>Complains about repeated delays but gives little specific flight context.</t>
+  </si>
+  <si>
+    <t>no actionable issue stated.</t>
+  </si>
+  <si>
+    <t>Primary question is baggage allowance; OneWorld Sapphire status is relevant secondary context.</t>
+  </si>
+  <si>
+    <t>Complaint-form/alternative complaint-submission method; website/app technical issue is not a v1 intent.</t>
+  </si>
+  <si>
+    <t>Negative customer-service experience stated without a specific actionable issue.</t>
+  </si>
+  <si>
+    <t>Passenger paperwork/documentation issue; no existing v1 intent clearly covers it.</t>
+  </si>
+  <si>
+    <t>Airport security/PreCheck complaint; no clear v1 intent covers security screening.</t>
+  </si>
+  <si>
+    <t>Positive travel/aviation commentary without a support request.</t>
+  </si>
+  <si>
+    <t>Complaint about itinerary/flight description at booking.</t>
+  </si>
+  <si>
+    <t>off to @46163 !! / Starting things off right with champagne in a plastic cup! Thanks @AmericanAir</t>
+  </si>
+  <si>
+    <t>couldnot understand</t>
+  </si>
+  <si>
+    <t>New-service announcement/travel information; no support intent fits.</t>
+  </si>
+  <si>
+    <t>Admirals Club/quiet-room complaint; lounge experience.</t>
+  </si>
+  <si>
+    <t>General negative complaint without a specific actionable request.</t>
+  </si>
+  <si>
+    <t>Explicitly asks why the flight is delayed.</t>
+  </si>
+  <si>
+    <t>Pet-related ticket/payment process; taxonomy boundary is unclear.</t>
+  </si>
+  <si>
+    <t>Stroller/gate-check issue is baggage-related.</t>
+  </si>
+  <si>
+    <t>Priority/boarding policy request involving connecting passengers.</t>
+  </si>
+  <si>
+    <t>Thanks agents for helping them get home.</t>
+  </si>
+  <si>
+    <t>Free upgrade is the concrete issue; praise/thanks is incidental.</t>
+  </si>
+  <si>
+    <t>Lost luggage/baggage claim and eventual delivery.</t>
+  </si>
+  <si>
+    <t>Sitting on runway for an hour.</t>
+  </si>
+  <si>
+    <t>Cancelled flight/rebooking plus missing miles information.</t>
+  </si>
+  <si>
+    <t>nothing specified properly</t>
+  </si>
+  <si>
+    <t>Trouble contacting American via phone/Skype; no v1 intent clearly covers it.</t>
+  </si>
+  <si>
+    <t>Complaint about aircraft/cabin and lack of first class; cabin-class issue.</t>
+  </si>
+  <si>
+    <t>Complaint about someone being downgraded from an upgrade.</t>
+  </si>
+  <si>
+    <t>nothing specified clearly</t>
+  </si>
+  <si>
+    <t>Carry-on check-in dispute; also complains about customer service.</t>
+  </si>
+  <si>
+    <t>Double charge for carry-on plus customer-service complaint.</t>
+  </si>
+  <si>
+    <t>not sure about this is correct</t>
+  </si>
+  <si>
+    <t>In-flight Wi-Fi unavailable; no current v1 intent covers this.</t>
+  </si>
+  <si>
+    <t>Multi-year offer/compensation issue does not clearly fit v1.</t>
+  </si>
+  <si>
+    <t>cant understand the message</t>
+  </si>
+  <si>
+    <t>not sure about it</t>
+  </si>
+  <si>
+    <t>Strongly implies a travel delay/disruption, but exact cause isn't stated.</t>
+  </si>
+  <si>
+    <t>Flight already listed as delayed; sarcastic wording.</t>
+  </si>
+  <si>
+    <t>Direct praise of flight attendant Josh.</t>
+  </si>
+  <si>
+    <t>don’t understand the clear message</t>
+  </si>
+  <si>
+    <t>message is not specifying any cause</t>
+  </si>
+  <si>
+    <t>Honeymoon/travel experience ruined; exact issue unclear</t>
+  </si>
+  <si>
+    <t>Flight changed + voucher/compensation issue</t>
+  </si>
+  <si>
+    <t>not sure about the answer</t>
+  </si>
+  <si>
+    <t>Cancelled flights + asking about refund</t>
+  </si>
+  <si>
+    <t>didn’t understand the message much</t>
+  </si>
+  <si>
+    <t>Major delay + first-class lounge access complaint</t>
+  </si>
+  <si>
+    <t>Asking about upgrade process</t>
+  </si>
+  <si>
+    <t>fligh_delay</t>
+  </si>
+  <si>
+    <t>Wants to know whether flight will operate and whether cancellation/refund is possible</t>
+  </si>
+  <si>
+    <t>not sure about the  message</t>
+  </si>
+  <si>
+    <t>baggae</t>
+  </si>
+  <si>
+    <t>Carry-on charge + rude gate agents + refund</t>
+  </si>
+  <si>
+    <t>General complaint about losing a First Class customer</t>
+  </si>
+  <si>
+    <t>Upgrade list/status/elite eligibility</t>
+  </si>
+  <si>
+    <t>Complaint about airline fees/charges</t>
+  </si>
+  <si>
+    <t>Paid for upgrade but seated behind open First Class seats</t>
+  </si>
+  <si>
+    <t>Admirals Club experience/food complaint</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1534,6 +1834,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1877,9 +2182,16 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2236,9 +2548,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78956FB4-83C4-4B81-8786-8036E0E87EFC}">
   <dimension ref="A1:L149"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="6.88671875" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" customWidth="1"/>
+    <col min="5" max="5" width="8.77734375" customWidth="1"/>
+    <col min="6" max="6" width="208" style="2" customWidth="1"/>
+    <col min="7" max="7" width="25.44140625" customWidth="1"/>
+    <col min="8" max="8" width="22.109375" customWidth="1"/>
+    <col min="9" max="9" width="17.77734375" customWidth="1"/>
+    <col min="10" max="10" width="13.33203125" customWidth="1"/>
+    <col min="11" max="11" width="15.77734375" customWidth="1"/>
+    <col min="12" max="12" width="91.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2254,7 +2580,7 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" t="s">
@@ -2276,7 +2602,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -2292,11 +2618,17 @@
       <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>457</v>
+      </c>
+      <c r="I2" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2312,11 +2644,17 @@
       <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>459</v>
+      </c>
+      <c r="I3" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -2332,11 +2670,23 @@
       <c r="E4" t="s">
         <v>14</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>460</v>
+      </c>
+      <c r="I4" t="s">
+        <v>461</v>
+      </c>
+      <c r="K4" t="s">
+        <v>462</v>
+      </c>
+      <c r="L4" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -2352,11 +2702,23 @@
       <c r="E5" t="s">
         <v>14</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>464</v>
+      </c>
+      <c r="I5" t="s">
+        <v>461</v>
+      </c>
+      <c r="K5" t="s">
+        <v>462</v>
+      </c>
+      <c r="L5" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -2372,11 +2734,26 @@
       <c r="E6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>459</v>
+      </c>
+      <c r="H6" t="s">
+        <v>466</v>
+      </c>
+      <c r="I6" t="s">
+        <v>461</v>
+      </c>
+      <c r="K6" t="s">
+        <v>462</v>
+      </c>
+      <c r="L6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -2392,11 +2769,23 @@
       <c r="E7" t="s">
         <v>14</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G7" t="s">
+        <v>459</v>
+      </c>
+      <c r="H7" t="s">
+        <v>466</v>
+      </c>
+      <c r="I7" t="s">
+        <v>458</v>
+      </c>
+      <c r="L7" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -2412,11 +2801,17 @@
       <c r="E8" t="s">
         <v>14</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G8" t="s">
+        <v>459</v>
+      </c>
+      <c r="I8" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -2432,11 +2827,23 @@
       <c r="E9" t="s">
         <v>14</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>468</v>
+      </c>
+      <c r="I9" t="s">
+        <v>461</v>
+      </c>
+      <c r="K9" t="s">
+        <v>462</v>
+      </c>
+      <c r="L9" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -2452,11 +2859,17 @@
       <c r="E10" t="s">
         <v>14</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G10" t="s">
+        <v>464</v>
+      </c>
+      <c r="I10" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -2472,11 +2885,17 @@
       <c r="E11" t="s">
         <v>14</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>468</v>
+      </c>
+      <c r="I11" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -2492,11 +2911,26 @@
       <c r="E12" t="s">
         <v>14</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G12" t="s">
+        <v>457</v>
+      </c>
+      <c r="I12" t="s">
+        <v>461</v>
+      </c>
+      <c r="J12" t="s">
+        <v>462</v>
+      </c>
+      <c r="K12" t="s">
+        <v>462</v>
+      </c>
+      <c r="L12" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" t="s">
         <v>46</v>
       </c>
@@ -2512,11 +2946,17 @@
       <c r="E13" t="s">
         <v>14</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G13" t="s">
+        <v>472</v>
+      </c>
+      <c r="I13" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -2532,11 +2972,26 @@
       <c r="E14" t="s">
         <v>14</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G14" t="s">
+        <v>464</v>
+      </c>
+      <c r="I14" t="s">
+        <v>473</v>
+      </c>
+      <c r="J14" t="s">
+        <v>462</v>
+      </c>
+      <c r="K14" t="s">
+        <v>462</v>
+      </c>
+      <c r="L14" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" t="s">
         <v>52</v>
       </c>
@@ -2552,11 +3007,17 @@
       <c r="E15" t="s">
         <v>14</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G15" t="s">
+        <v>457</v>
+      </c>
+      <c r="I15" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" t="s">
         <v>55</v>
       </c>
@@ -2572,11 +3033,23 @@
       <c r="E16" t="s">
         <v>14</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G16" t="s">
+        <v>468</v>
+      </c>
+      <c r="I16" t="s">
+        <v>461</v>
+      </c>
+      <c r="K16" t="s">
+        <v>462</v>
+      </c>
+      <c r="L16" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17" t="s">
         <v>58</v>
       </c>
@@ -2592,11 +3065,29 @@
       <c r="E17" t="s">
         <v>14</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G17" t="s">
+        <v>459</v>
+      </c>
+      <c r="H17" t="s">
+        <v>476</v>
+      </c>
+      <c r="I17" t="s">
+        <v>461</v>
+      </c>
+      <c r="J17" t="s">
+        <v>462</v>
+      </c>
+      <c r="K17" t="s">
+        <v>462</v>
+      </c>
+      <c r="L17" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
       <c r="A18" t="s">
         <v>61</v>
       </c>
@@ -2612,11 +3103,17 @@
       <c r="E18" t="s">
         <v>14</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="2" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G18" t="s">
+        <v>478</v>
+      </c>
+      <c r="I18" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19" t="s">
         <v>64</v>
       </c>
@@ -2632,11 +3129,17 @@
       <c r="E19" t="s">
         <v>14</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19" t="s">
+        <v>472</v>
+      </c>
+      <c r="I19" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
       <c r="A20" t="s">
         <v>67</v>
       </c>
@@ -2652,11 +3155,20 @@
       <c r="E20" t="s">
         <v>14</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G20" t="s">
+        <v>479</v>
+      </c>
+      <c r="I20" t="s">
+        <v>458</v>
+      </c>
+      <c r="L20" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
       <c r="A21" t="s">
         <v>70</v>
       </c>
@@ -2672,11 +3184,23 @@
       <c r="E21" t="s">
         <v>14</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G21" t="s">
+        <v>459</v>
+      </c>
+      <c r="H21" t="s">
+        <v>481</v>
+      </c>
+      <c r="I21" t="s">
+        <v>458</v>
+      </c>
+      <c r="L21" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -2692,11 +3216,23 @@
       <c r="E22" t="s">
         <v>14</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G22" t="s">
+        <v>479</v>
+      </c>
+      <c r="I22" t="s">
+        <v>458</v>
+      </c>
+      <c r="K22" t="s">
+        <v>462</v>
+      </c>
+      <c r="L22" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
       <c r="A23" t="s">
         <v>76</v>
       </c>
@@ -2712,11 +3248,17 @@
       <c r="E23" t="s">
         <v>14</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G23" t="s">
+        <v>466</v>
+      </c>
+      <c r="I23" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
       <c r="A24" t="s">
         <v>79</v>
       </c>
@@ -2732,11 +3274,20 @@
       <c r="E24" t="s">
         <v>14</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G24" t="s">
+        <v>479</v>
+      </c>
+      <c r="I24" t="s">
+        <v>458</v>
+      </c>
+      <c r="L24" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
       <c r="A25" t="s">
         <v>82</v>
       </c>
@@ -2752,11 +3303,17 @@
       <c r="E25" t="s">
         <v>14</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="2" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G25" t="s">
+        <v>485</v>
+      </c>
+      <c r="I25" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
       <c r="A26" t="s">
         <v>85</v>
       </c>
@@ -2772,11 +3329,17 @@
       <c r="E26" t="s">
         <v>14</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G26" t="s">
+        <v>464</v>
+      </c>
+      <c r="I26" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
       <c r="A27" t="s">
         <v>88</v>
       </c>
@@ -2792,11 +3355,17 @@
       <c r="E27" t="s">
         <v>14</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G27" t="s">
+        <v>481</v>
+      </c>
+      <c r="I27" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
       <c r="A28" t="s">
         <v>91</v>
       </c>
@@ -2812,11 +3381,17 @@
       <c r="E28" t="s">
         <v>14</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28" t="s">
+        <v>457</v>
+      </c>
+      <c r="I28" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
       <c r="A29" t="s">
         <v>94</v>
       </c>
@@ -2832,11 +3407,29 @@
       <c r="E29" t="s">
         <v>14</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G29" t="s">
+        <v>486</v>
+      </c>
+      <c r="H29" t="s">
+        <v>464</v>
+      </c>
+      <c r="I29" t="s">
+        <v>461</v>
+      </c>
+      <c r="J29" t="s">
+        <v>462</v>
+      </c>
+      <c r="K29" t="s">
+        <v>462</v>
+      </c>
+      <c r="L29" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
       <c r="A30" t="s">
         <v>97</v>
       </c>
@@ -2852,11 +3445,20 @@
       <c r="E30" t="s">
         <v>14</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="2" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G30" t="s">
+        <v>479</v>
+      </c>
+      <c r="I30" t="s">
+        <v>458</v>
+      </c>
+      <c r="L30" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
       <c r="A31" t="s">
         <v>100</v>
       </c>
@@ -2872,11 +3474,17 @@
       <c r="E31" t="s">
         <v>14</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G31" t="s">
+        <v>464</v>
+      </c>
+      <c r="I31" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
       <c r="A32" t="s">
         <v>103</v>
       </c>
@@ -2892,11 +3500,17 @@
       <c r="E32" t="s">
         <v>14</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G32" t="s">
+        <v>464</v>
+      </c>
+      <c r="I32" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
       <c r="A33" t="s">
         <v>106</v>
       </c>
@@ -2912,11 +3526,23 @@
       <c r="E33" t="s">
         <v>14</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G33" t="s">
+        <v>460</v>
+      </c>
+      <c r="I33" t="s">
+        <v>473</v>
+      </c>
+      <c r="K33" t="s">
+        <v>462</v>
+      </c>
+      <c r="L33" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
       <c r="A34" t="s">
         <v>109</v>
       </c>
@@ -2932,11 +3558,17 @@
       <c r="E34" t="s">
         <v>14</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="2" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G34" t="s">
+        <v>457</v>
+      </c>
+      <c r="I34" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
       <c r="A35" t="s">
         <v>112</v>
       </c>
@@ -2952,11 +3584,23 @@
       <c r="E35" t="s">
         <v>14</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G35" t="s">
+        <v>472</v>
+      </c>
+      <c r="I35" t="s">
+        <v>458</v>
+      </c>
+      <c r="K35" t="s">
+        <v>462</v>
+      </c>
+      <c r="L35" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
       <c r="A36" t="s">
         <v>115</v>
       </c>
@@ -2972,11 +3616,17 @@
       <c r="E36" t="s">
         <v>14</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G36" t="s">
+        <v>459</v>
+      </c>
+      <c r="I36" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
       <c r="A37" t="s">
         <v>118</v>
       </c>
@@ -2992,11 +3642,17 @@
       <c r="E37" t="s">
         <v>14</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="2" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G37" t="s">
+        <v>468</v>
+      </c>
+      <c r="I37" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
       <c r="A38" t="s">
         <v>121</v>
       </c>
@@ -3012,11 +3668,17 @@
       <c r="E38" t="s">
         <v>14</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="2" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38" t="s">
+        <v>459</v>
+      </c>
+      <c r="I38" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
       <c r="A39" t="s">
         <v>124</v>
       </c>
@@ -3032,11 +3694,26 @@
       <c r="E39" t="s">
         <v>14</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39" t="s">
+        <v>459</v>
+      </c>
+      <c r="H39" t="s">
+        <v>486</v>
+      </c>
+      <c r="I39" t="s">
+        <v>458</v>
+      </c>
+      <c r="J39" t="s">
+        <v>462</v>
+      </c>
+      <c r="L39" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
       <c r="A40" t="s">
         <v>127</v>
       </c>
@@ -3052,11 +3729,26 @@
       <c r="E40" t="s">
         <v>14</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G40" t="s">
+        <v>485</v>
+      </c>
+      <c r="I40" t="s">
+        <v>461</v>
+      </c>
+      <c r="J40" t="s">
+        <v>462</v>
+      </c>
+      <c r="K40" t="s">
+        <v>462</v>
+      </c>
+      <c r="L40" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
       <c r="A41" t="s">
         <v>130</v>
       </c>
@@ -3072,11 +3764,20 @@
       <c r="E41" t="s">
         <v>14</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" s="2" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G41" t="s">
+        <v>464</v>
+      </c>
+      <c r="I41" t="s">
+        <v>458</v>
+      </c>
+      <c r="L41" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
       <c r="A42" t="s">
         <v>133</v>
       </c>
@@ -3092,11 +3793,17 @@
       <c r="E42" t="s">
         <v>14</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G42" t="s">
+        <v>485</v>
+      </c>
+      <c r="I42" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12">
       <c r="A43" t="s">
         <v>136</v>
       </c>
@@ -3112,11 +3819,17 @@
       <c r="E43" t="s">
         <v>14</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G43" t="s">
+        <v>478</v>
+      </c>
+      <c r="I43" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12">
       <c r="A44" t="s">
         <v>139</v>
       </c>
@@ -3132,11 +3845,17 @@
       <c r="E44" t="s">
         <v>14</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F44" s="2" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G44" t="s">
+        <v>457</v>
+      </c>
+      <c r="I44" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12">
       <c r="A45" t="s">
         <v>142</v>
       </c>
@@ -3152,11 +3871,23 @@
       <c r="E45" t="s">
         <v>14</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" s="2" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G45" t="s">
+        <v>478</v>
+      </c>
+      <c r="I45" t="s">
+        <v>458</v>
+      </c>
+      <c r="K45" t="s">
+        <v>462</v>
+      </c>
+      <c r="L45" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12">
       <c r="A46" t="s">
         <v>145</v>
       </c>
@@ -3172,11 +3903,26 @@
       <c r="E46" t="s">
         <v>14</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="2" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G46" t="s">
+        <v>459</v>
+      </c>
+      <c r="I46" t="s">
+        <v>461</v>
+      </c>
+      <c r="J46" t="s">
+        <v>462</v>
+      </c>
+      <c r="K46" t="s">
+        <v>462</v>
+      </c>
+      <c r="L46" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12">
       <c r="A47" t="s">
         <v>148</v>
       </c>
@@ -3192,11 +3938,17 @@
       <c r="E47" t="s">
         <v>14</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G47" t="s">
+        <v>459</v>
+      </c>
+      <c r="I47" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12">
       <c r="A48" t="s">
         <v>151</v>
       </c>
@@ -3212,11 +3964,23 @@
       <c r="E48" t="s">
         <v>14</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48" s="2" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G48" t="s">
+        <v>459</v>
+      </c>
+      <c r="I48" t="s">
+        <v>458</v>
+      </c>
+      <c r="K48" t="s">
+        <v>462</v>
+      </c>
+      <c r="L48" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12">
       <c r="A49" t="s">
         <v>154</v>
       </c>
@@ -3232,11 +3996,20 @@
       <c r="E49" t="s">
         <v>14</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F49" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G49" t="s">
+        <v>479</v>
+      </c>
+      <c r="I49" t="s">
+        <v>458</v>
+      </c>
+      <c r="L49" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12">
       <c r="A50" t="s">
         <v>157</v>
       </c>
@@ -3252,11 +4025,29 @@
       <c r="E50" t="s">
         <v>14</v>
       </c>
-      <c r="F50" t="s">
+      <c r="F50" s="2" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G50" t="s">
+        <v>478</v>
+      </c>
+      <c r="H50" t="s">
+        <v>464</v>
+      </c>
+      <c r="I50" t="s">
+        <v>461</v>
+      </c>
+      <c r="J50" t="s">
+        <v>462</v>
+      </c>
+      <c r="K50" t="s">
+        <v>462</v>
+      </c>
+      <c r="L50" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12">
       <c r="A51" t="s">
         <v>160</v>
       </c>
@@ -3272,11 +4063,26 @@
       <c r="E51" t="s">
         <v>14</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F51" s="2" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G51" t="s">
+        <v>481</v>
+      </c>
+      <c r="I51" t="s">
+        <v>461</v>
+      </c>
+      <c r="J51" t="s">
+        <v>462</v>
+      </c>
+      <c r="K51" t="s">
+        <v>462</v>
+      </c>
+      <c r="L51" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12">
       <c r="A52" t="s">
         <v>163</v>
       </c>
@@ -3292,11 +4098,17 @@
       <c r="E52" t="s">
         <v>14</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F52" s="2" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G52" t="s">
+        <v>466</v>
+      </c>
+      <c r="I52" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12">
       <c r="A53" t="s">
         <v>166</v>
       </c>
@@ -3312,11 +4124,23 @@
       <c r="E53" t="s">
         <v>14</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F53" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G53" t="s">
+        <v>457</v>
+      </c>
+      <c r="I53" t="s">
+        <v>461</v>
+      </c>
+      <c r="K53" t="s">
+        <v>462</v>
+      </c>
+      <c r="L53" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12">
       <c r="A54" t="s">
         <v>169</v>
       </c>
@@ -3332,11 +4156,17 @@
       <c r="E54" t="s">
         <v>14</v>
       </c>
-      <c r="F54" t="s">
+      <c r="F54" s="2" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G54" t="s">
+        <v>481</v>
+      </c>
+      <c r="I54" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12">
       <c r="A55" t="s">
         <v>172</v>
       </c>
@@ -3352,11 +4182,23 @@
       <c r="E55" t="s">
         <v>14</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F55" s="2" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G55" t="s">
+        <v>459</v>
+      </c>
+      <c r="I55" t="s">
+        <v>461</v>
+      </c>
+      <c r="K55" t="s">
+        <v>462</v>
+      </c>
+      <c r="L55" s="3" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12">
       <c r="A56" t="s">
         <v>175</v>
       </c>
@@ -3372,11 +4214,20 @@
       <c r="E56" t="s">
         <v>14</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F56" s="2" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G56" t="s">
+        <v>479</v>
+      </c>
+      <c r="I56" t="s">
+        <v>458</v>
+      </c>
+      <c r="L56" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12">
       <c r="A57" t="s">
         <v>178</v>
       </c>
@@ -3392,11 +4243,17 @@
       <c r="E57" t="s">
         <v>14</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F57" s="2" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G57" t="s">
+        <v>459</v>
+      </c>
+      <c r="I57" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12">
       <c r="A58" t="s">
         <v>181</v>
       </c>
@@ -3412,11 +4269,29 @@
       <c r="E58" t="s">
         <v>14</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F58" s="2" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G58" t="s">
+        <v>466</v>
+      </c>
+      <c r="H58" t="s">
+        <v>485</v>
+      </c>
+      <c r="I58" t="s">
+        <v>458</v>
+      </c>
+      <c r="J58" t="s">
+        <v>462</v>
+      </c>
+      <c r="K58" t="s">
+        <v>462</v>
+      </c>
+      <c r="L58" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12">
       <c r="A59" t="s">
         <v>184</v>
       </c>
@@ -3432,11 +4307,23 @@
       <c r="E59" t="s">
         <v>14</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F59" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G59" t="s">
+        <v>460</v>
+      </c>
+      <c r="I59" t="s">
+        <v>458</v>
+      </c>
+      <c r="K59" t="s">
+        <v>462</v>
+      </c>
+      <c r="L59" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12">
       <c r="A60" t="s">
         <v>187</v>
       </c>
@@ -3452,11 +4339,23 @@
       <c r="E60" t="s">
         <v>14</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F60" s="2" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G60" t="s">
+        <v>468</v>
+      </c>
+      <c r="I60" t="s">
+        <v>461</v>
+      </c>
+      <c r="K60" t="s">
+        <v>462</v>
+      </c>
+      <c r="L60" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12">
       <c r="A61" t="s">
         <v>190</v>
       </c>
@@ -3472,11 +4371,23 @@
       <c r="E61" t="s">
         <v>14</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F61" s="2" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G61" t="s">
+        <v>460</v>
+      </c>
+      <c r="I61" t="s">
+        <v>461</v>
+      </c>
+      <c r="K61" t="s">
+        <v>462</v>
+      </c>
+      <c r="L61" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12">
       <c r="A62" t="s">
         <v>193</v>
       </c>
@@ -3492,11 +4403,17 @@
       <c r="E62" t="s">
         <v>14</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F62" s="2" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G62" t="s">
+        <v>459</v>
+      </c>
+      <c r="I62" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12">
       <c r="A63" t="s">
         <v>196</v>
       </c>
@@ -3512,11 +4429,26 @@
       <c r="E63" t="s">
         <v>14</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F63" s="2" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G63" t="s">
+        <v>460</v>
+      </c>
+      <c r="I63" t="s">
+        <v>458</v>
+      </c>
+      <c r="J63" t="s">
+        <v>462</v>
+      </c>
+      <c r="K63" t="s">
+        <v>462</v>
+      </c>
+      <c r="L63" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12">
       <c r="A64" t="s">
         <v>199</v>
       </c>
@@ -3532,11 +4464,17 @@
       <c r="E64" t="s">
         <v>14</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F64" s="2" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G64" t="s">
+        <v>457</v>
+      </c>
+      <c r="I64" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12">
       <c r="A65" t="s">
         <v>202</v>
       </c>
@@ -3552,11 +4490,23 @@
       <c r="E65" t="s">
         <v>14</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F65" s="2" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G65" t="s">
+        <v>460</v>
+      </c>
+      <c r="I65" t="s">
+        <v>461</v>
+      </c>
+      <c r="K65" t="s">
+        <v>462</v>
+      </c>
+      <c r="L65" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12">
       <c r="A66" t="s">
         <v>205</v>
       </c>
@@ -3572,11 +4522,20 @@
       <c r="E66" t="s">
         <v>14</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F66" s="2" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G66" t="s">
+        <v>464</v>
+      </c>
+      <c r="I66" t="s">
+        <v>458</v>
+      </c>
+      <c r="L66" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12">
       <c r="A67" t="s">
         <v>208</v>
       </c>
@@ -3592,16 +4551,28 @@
       <c r="E67" t="s">
         <v>14</v>
       </c>
-      <c r="F67" t="s">
+      <c r="F67" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="G67" t="s">
+        <v>460</v>
+      </c>
+      <c r="I67" t="s">
+        <v>458</v>
+      </c>
+      <c r="K67" t="s">
+        <v>462</v>
+      </c>
+      <c r="L67" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12">
+      <c r="A68" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
+      <c r="B68" t="s">
         <v>211</v>
-      </c>
-      <c r="B68" t="s">
-        <v>212</v>
       </c>
       <c r="C68">
         <v>2413154</v>
@@ -3612,16 +4583,28 @@
       <c r="E68" t="s">
         <v>14</v>
       </c>
-      <c r="F68" t="s">
+      <c r="F68" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="G68" t="s">
+        <v>460</v>
+      </c>
+      <c r="I68" t="s">
+        <v>458</v>
+      </c>
+      <c r="K68" t="s">
+        <v>462</v>
+      </c>
+      <c r="L68" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12">
+      <c r="A69" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
+      <c r="B69" t="s">
         <v>214</v>
-      </c>
-      <c r="B69" t="s">
-        <v>215</v>
       </c>
       <c r="C69">
         <v>248276</v>
@@ -3632,16 +4615,31 @@
       <c r="E69" t="s">
         <v>14</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F69" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="G69" t="s">
+        <v>485</v>
+      </c>
+      <c r="I69" t="s">
+        <v>461</v>
+      </c>
+      <c r="J69" t="s">
+        <v>462</v>
+      </c>
+      <c r="K69" t="s">
+        <v>462</v>
+      </c>
+      <c r="L69" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12">
+      <c r="A70" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
+      <c r="B70" t="s">
         <v>217</v>
-      </c>
-      <c r="B70" t="s">
-        <v>218</v>
       </c>
       <c r="C70">
         <v>2584631</v>
@@ -3652,16 +4650,22 @@
       <c r="E70" t="s">
         <v>14</v>
       </c>
-      <c r="F70" t="s">
+      <c r="F70" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G70" t="s">
+        <v>457</v>
+      </c>
+      <c r="I70" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12">
+      <c r="A71" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
+      <c r="B71" t="s">
         <v>220</v>
-      </c>
-      <c r="B71" t="s">
-        <v>221</v>
       </c>
       <c r="C71">
         <v>2621395</v>
@@ -3672,16 +4676,25 @@
       <c r="E71" t="s">
         <v>14</v>
       </c>
-      <c r="F71" t="s">
+      <c r="F71" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="G71" t="s">
+        <v>468</v>
+      </c>
+      <c r="I71" t="s">
+        <v>458</v>
+      </c>
+      <c r="L71" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12">
+      <c r="A72" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
+      <c r="B72" t="s">
         <v>223</v>
-      </c>
-      <c r="B72" t="s">
-        <v>224</v>
       </c>
       <c r="C72">
         <v>2710229</v>
@@ -3692,16 +4705,25 @@
       <c r="E72" t="s">
         <v>14</v>
       </c>
-      <c r="F72" t="s">
+      <c r="F72" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="G72" t="s">
+        <v>459</v>
+      </c>
+      <c r="I72" t="s">
+        <v>458</v>
+      </c>
+      <c r="L72" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12">
+      <c r="A73" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
+      <c r="B73" t="s">
         <v>226</v>
-      </c>
-      <c r="B73" t="s">
-        <v>227</v>
       </c>
       <c r="C73">
         <v>2721563</v>
@@ -3712,16 +4734,22 @@
       <c r="E73" t="s">
         <v>14</v>
       </c>
-      <c r="F73" t="s">
+      <c r="F73" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="G73" t="s">
+        <v>459</v>
+      </c>
+      <c r="I73" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12">
+      <c r="A74" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
+      <c r="B74" t="s">
         <v>229</v>
-      </c>
-      <c r="B74" t="s">
-        <v>230</v>
       </c>
       <c r="C74">
         <v>2729549</v>
@@ -3732,16 +4760,31 @@
       <c r="E74" t="s">
         <v>14</v>
       </c>
-      <c r="F74" t="s">
+      <c r="F74" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="G74" t="s">
+        <v>464</v>
+      </c>
+      <c r="I74" t="s">
+        <v>461</v>
+      </c>
+      <c r="J74" t="s">
+        <v>462</v>
+      </c>
+      <c r="K74" t="s">
+        <v>462</v>
+      </c>
+      <c r="L74" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12">
+      <c r="A75" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
+      <c r="B75" t="s">
         <v>232</v>
-      </c>
-      <c r="B75" t="s">
-        <v>233</v>
       </c>
       <c r="C75">
         <v>2748732</v>
@@ -3752,16 +4795,22 @@
       <c r="E75" t="s">
         <v>14</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F75" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="G75" t="s">
+        <v>460</v>
+      </c>
+      <c r="I75" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12">
+      <c r="A76" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
+      <c r="B76" t="s">
         <v>235</v>
-      </c>
-      <c r="B76" t="s">
-        <v>236</v>
       </c>
       <c r="C76">
         <v>2755129</v>
@@ -3772,16 +4821,28 @@
       <c r="E76" t="s">
         <v>14</v>
       </c>
-      <c r="F76" t="s">
+      <c r="F76" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="G76" t="s">
+        <v>466</v>
+      </c>
+      <c r="I76" t="s">
+        <v>458</v>
+      </c>
+      <c r="K76" t="s">
+        <v>462</v>
+      </c>
+      <c r="L76" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12">
+      <c r="A77" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
+      <c r="B77" t="s">
         <v>238</v>
-      </c>
-      <c r="B77" t="s">
-        <v>239</v>
       </c>
       <c r="C77">
         <v>2783717</v>
@@ -3792,16 +4853,22 @@
       <c r="E77" t="s">
         <v>14</v>
       </c>
-      <c r="F77" t="s">
+      <c r="F77" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="G77" t="s">
+        <v>459</v>
+      </c>
+      <c r="I77" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12">
+      <c r="A78" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
+      <c r="B78" t="s">
         <v>241</v>
-      </c>
-      <c r="B78" t="s">
-        <v>242</v>
       </c>
       <c r="C78">
         <v>2784936</v>
@@ -3812,16 +4879,22 @@
       <c r="E78" t="s">
         <v>14</v>
       </c>
-      <c r="F78" t="s">
+      <c r="F78" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="G78" t="s">
+        <v>464</v>
+      </c>
+      <c r="I78" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12">
+      <c r="A79" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
+      <c r="B79" t="s">
         <v>244</v>
-      </c>
-      <c r="B79" t="s">
-        <v>245</v>
       </c>
       <c r="C79">
         <v>27966</v>
@@ -3832,16 +4905,25 @@
       <c r="E79" t="s">
         <v>14</v>
       </c>
-      <c r="F79" t="s">
+      <c r="F79" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G79" t="s">
+        <v>457</v>
+      </c>
+      <c r="I79" t="s">
+        <v>458</v>
+      </c>
+      <c r="L79" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12">
+      <c r="A80" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
+      <c r="B80" t="s">
         <v>247</v>
-      </c>
-      <c r="B80" t="s">
-        <v>248</v>
       </c>
       <c r="C80">
         <v>2804658</v>
@@ -3852,16 +4934,31 @@
       <c r="E80" t="s">
         <v>14</v>
       </c>
-      <c r="F80" t="s">
+      <c r="F80" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="G80" t="s">
+        <v>481</v>
+      </c>
+      <c r="I80" t="s">
+        <v>461</v>
+      </c>
+      <c r="J80" t="s">
+        <v>462</v>
+      </c>
+      <c r="K80" t="s">
+        <v>462</v>
+      </c>
+      <c r="L80" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12">
+      <c r="A81" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
+      <c r="B81" t="s">
         <v>250</v>
-      </c>
-      <c r="B81" t="s">
-        <v>251</v>
       </c>
       <c r="C81">
         <v>2807954</v>
@@ -3872,16 +4969,34 @@
       <c r="E81" t="s">
         <v>14</v>
       </c>
-      <c r="F81" t="s">
+      <c r="F81" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="G81" t="s">
+        <v>459</v>
+      </c>
+      <c r="H81" t="s">
+        <v>485</v>
+      </c>
+      <c r="I81" t="s">
+        <v>461</v>
+      </c>
+      <c r="J81" t="s">
+        <v>462</v>
+      </c>
+      <c r="K81" t="s">
+        <v>462</v>
+      </c>
+      <c r="L81" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12">
+      <c r="A82" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
+      <c r="B82" t="s">
         <v>253</v>
-      </c>
-      <c r="B82" t="s">
-        <v>254</v>
       </c>
       <c r="C82">
         <v>2814078</v>
@@ -3892,16 +5007,25 @@
       <c r="E82" t="s">
         <v>14</v>
       </c>
-      <c r="F82" t="s">
+      <c r="F82" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="G82" t="s">
+        <v>459</v>
+      </c>
+      <c r="I82" t="s">
+        <v>458</v>
+      </c>
+      <c r="K82" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12">
+      <c r="A83" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
+      <c r="B83" t="s">
         <v>256</v>
-      </c>
-      <c r="B83" t="s">
-        <v>257</v>
       </c>
       <c r="C83">
         <v>2815163</v>
@@ -3912,16 +5036,31 @@
       <c r="E83" t="s">
         <v>14</v>
       </c>
-      <c r="F83" t="s">
+      <c r="F83" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G83" t="s">
+        <v>478</v>
+      </c>
+      <c r="I83" t="s">
+        <v>461</v>
+      </c>
+      <c r="J83" t="s">
+        <v>462</v>
+      </c>
+      <c r="K83" t="s">
+        <v>462</v>
+      </c>
+      <c r="L83" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12">
+      <c r="A84" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
+      <c r="B84" t="s">
         <v>259</v>
-      </c>
-      <c r="B84" t="s">
-        <v>260</v>
       </c>
       <c r="C84">
         <v>2817529</v>
@@ -3932,16 +5071,25 @@
       <c r="E84" t="s">
         <v>14</v>
       </c>
-      <c r="F84" t="s">
+      <c r="F84" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="G84" t="s">
+        <v>466</v>
+      </c>
+      <c r="I84" t="s">
+        <v>458</v>
+      </c>
+      <c r="L84" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12">
+      <c r="A85" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
+      <c r="B85" t="s">
         <v>262</v>
-      </c>
-      <c r="B85" t="s">
-        <v>263</v>
       </c>
       <c r="C85">
         <v>2821385</v>
@@ -3952,16 +5100,25 @@
       <c r="E85" t="s">
         <v>14</v>
       </c>
-      <c r="F85" t="s">
+      <c r="F85" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G85" t="s">
+        <v>459</v>
+      </c>
+      <c r="I85" t="s">
+        <v>458</v>
+      </c>
+      <c r="L85" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12">
+      <c r="A86" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
+      <c r="B86" t="s">
         <v>265</v>
-      </c>
-      <c r="B86" t="s">
-        <v>266</v>
       </c>
       <c r="C86">
         <v>2841271</v>
@@ -3972,16 +5129,34 @@
       <c r="E86" t="s">
         <v>14</v>
       </c>
-      <c r="F86" t="s">
+      <c r="F86" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G86" t="s">
+        <v>486</v>
+      </c>
+      <c r="H86" t="s">
+        <v>485</v>
+      </c>
+      <c r="I86" t="s">
+        <v>461</v>
+      </c>
+      <c r="J86" t="s">
+        <v>462</v>
+      </c>
+      <c r="K86" t="s">
+        <v>462</v>
+      </c>
+      <c r="L86" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12">
+      <c r="A87" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
+      <c r="B87" t="s">
         <v>268</v>
-      </c>
-      <c r="B87" t="s">
-        <v>269</v>
       </c>
       <c r="C87">
         <v>2844796</v>
@@ -3992,16 +5167,22 @@
       <c r="E87" t="s">
         <v>14</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F87" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="G87" t="s">
+        <v>466</v>
+      </c>
+      <c r="I87" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12">
+      <c r="A88" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
+      <c r="B88" t="s">
         <v>271</v>
-      </c>
-      <c r="B88" t="s">
-        <v>272</v>
       </c>
       <c r="C88">
         <v>2863050</v>
@@ -4012,16 +5193,28 @@
       <c r="E88" t="s">
         <v>14</v>
       </c>
-      <c r="F88" t="s">
+      <c r="F88" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="G88" t="s">
+        <v>460</v>
+      </c>
+      <c r="I88" t="s">
+        <v>458</v>
+      </c>
+      <c r="K88" t="s">
+        <v>462</v>
+      </c>
+      <c r="L88" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12">
+      <c r="A89" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
+      <c r="B89" t="s">
         <v>274</v>
-      </c>
-      <c r="B89" t="s">
-        <v>275</v>
       </c>
       <c r="C89">
         <v>2924121</v>
@@ -4032,16 +5225,28 @@
       <c r="E89" t="s">
         <v>14</v>
       </c>
-      <c r="F89" t="s">
+      <c r="F89" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G89" t="s">
+        <v>460</v>
+      </c>
+      <c r="I89" t="s">
+        <v>458</v>
+      </c>
+      <c r="K89" t="s">
+        <v>462</v>
+      </c>
+      <c r="L89" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12">
+      <c r="A90" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
+      <c r="B90" t="s">
         <v>277</v>
-      </c>
-      <c r="B90" t="s">
-        <v>278</v>
       </c>
       <c r="C90">
         <v>2968550</v>
@@ -4052,16 +5257,31 @@
       <c r="E90" t="s">
         <v>14</v>
       </c>
-      <c r="F90" t="s">
+      <c r="F90" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="G90" t="s">
+        <v>478</v>
+      </c>
+      <c r="I90" t="s">
+        <v>461</v>
+      </c>
+      <c r="J90" t="s">
+        <v>462</v>
+      </c>
+      <c r="K90" t="s">
+        <v>462</v>
+      </c>
+      <c r="L90" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12">
+      <c r="A91" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
+      <c r="B91" t="s">
         <v>280</v>
-      </c>
-      <c r="B91" t="s">
-        <v>281</v>
       </c>
       <c r="C91">
         <v>298402</v>
@@ -4072,16 +5292,22 @@
       <c r="E91" t="s">
         <v>14</v>
       </c>
-      <c r="F91" t="s">
+      <c r="F91" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="G91" t="s">
+        <v>459</v>
+      </c>
+      <c r="I91" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12">
+      <c r="A92" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" t="s">
+      <c r="B92" t="s">
         <v>283</v>
-      </c>
-      <c r="B92" t="s">
-        <v>284</v>
       </c>
       <c r="C92">
         <v>307021</v>
@@ -4092,16 +5318,31 @@
       <c r="E92" t="s">
         <v>14</v>
       </c>
-      <c r="F92" t="s">
+      <c r="F92" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="G92" t="s">
+        <v>478</v>
+      </c>
+      <c r="I92" t="s">
+        <v>461</v>
+      </c>
+      <c r="J92" t="s">
+        <v>462</v>
+      </c>
+      <c r="K92" t="s">
+        <v>462</v>
+      </c>
+      <c r="L92" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12">
+      <c r="A93" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
+      <c r="B93" t="s">
         <v>286</v>
-      </c>
-      <c r="B93" t="s">
-        <v>287</v>
       </c>
       <c r="C93">
         <v>327144</v>
@@ -4112,16 +5353,22 @@
       <c r="E93" t="s">
         <v>14</v>
       </c>
-      <c r="F93" t="s">
+      <c r="F93" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="G93" t="s">
+        <v>457</v>
+      </c>
+      <c r="I93" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12">
+      <c r="A94" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
+      <c r="B94" t="s">
         <v>289</v>
-      </c>
-      <c r="B94" t="s">
-        <v>290</v>
       </c>
       <c r="C94">
         <v>347838</v>
@@ -4132,16 +5379,28 @@
       <c r="E94" t="s">
         <v>14</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F94" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="G94" t="s">
+        <v>460</v>
+      </c>
+      <c r="I94" t="s">
+        <v>458</v>
+      </c>
+      <c r="K94" t="s">
+        <v>462</v>
+      </c>
+      <c r="L94" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12">
+      <c r="A95" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
+      <c r="B95" t="s">
         <v>292</v>
-      </c>
-      <c r="B95" t="s">
-        <v>293</v>
       </c>
       <c r="C95">
         <v>398942</v>
@@ -4152,16 +5411,31 @@
       <c r="E95" t="s">
         <v>14</v>
       </c>
-      <c r="F95" t="s">
+      <c r="F95" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="G95" t="s">
+        <v>466</v>
+      </c>
+      <c r="I95" t="s">
+        <v>458</v>
+      </c>
+      <c r="J95" t="s">
+        <v>462</v>
+      </c>
+      <c r="K95" t="s">
+        <v>462</v>
+      </c>
+      <c r="L95" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12">
+      <c r="A96" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
+      <c r="B96" t="s">
         <v>295</v>
-      </c>
-      <c r="B96" t="s">
-        <v>296</v>
       </c>
       <c r="C96">
         <v>410199</v>
@@ -4172,16 +5446,22 @@
       <c r="E96" t="s">
         <v>14</v>
       </c>
-      <c r="F96" t="s">
+      <c r="F96" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="G96" t="s">
+        <v>466</v>
+      </c>
+      <c r="I96" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12">
+      <c r="A97" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
+      <c r="B97" t="s">
         <v>298</v>
-      </c>
-      <c r="B97" t="s">
-        <v>299</v>
       </c>
       <c r="C97">
         <v>415845</v>
@@ -4192,16 +5472,31 @@
       <c r="E97" t="s">
         <v>14</v>
       </c>
-      <c r="F97" t="s">
+      <c r="F97" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="G97" t="s">
+        <v>466</v>
+      </c>
+      <c r="I97" t="s">
+        <v>458</v>
+      </c>
+      <c r="J97" t="s">
+        <v>462</v>
+      </c>
+      <c r="K97" t="s">
+        <v>462</v>
+      </c>
+      <c r="L97" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12">
+      <c r="A98" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
+      <c r="B98" t="s">
         <v>301</v>
-      </c>
-      <c r="B98" t="s">
-        <v>302</v>
       </c>
       <c r="C98">
         <v>450985</v>
@@ -4212,16 +5507,22 @@
       <c r="E98" t="s">
         <v>14</v>
       </c>
-      <c r="F98" t="s">
+      <c r="F98" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="G98" t="s">
+        <v>459</v>
+      </c>
+      <c r="I98" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12">
+      <c r="A99" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
+      <c r="B99" t="s">
         <v>304</v>
-      </c>
-      <c r="B99" t="s">
-        <v>305</v>
       </c>
       <c r="C99">
         <v>46982</v>
@@ -4232,16 +5533,28 @@
       <c r="E99" t="s">
         <v>14</v>
       </c>
-      <c r="F99" t="s">
+      <c r="F99" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="G99" t="s">
+        <v>457</v>
+      </c>
+      <c r="I99" t="s">
+        <v>458</v>
+      </c>
+      <c r="K99" t="s">
+        <v>462</v>
+      </c>
+      <c r="L99" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12">
+      <c r="A100" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
+      <c r="B100" t="s">
         <v>307</v>
-      </c>
-      <c r="B100" t="s">
-        <v>308</v>
       </c>
       <c r="C100">
         <v>522782</v>
@@ -4252,16 +5565,28 @@
       <c r="E100" t="s">
         <v>14</v>
       </c>
-      <c r="F100" t="s">
+      <c r="F100" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G100" t="s">
+        <v>479</v>
+      </c>
+      <c r="I100" t="s">
+        <v>458</v>
+      </c>
+      <c r="K100" t="s">
+        <v>462</v>
+      </c>
+      <c r="L100" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12">
+      <c r="A101" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
+      <c r="B101" t="s">
         <v>310</v>
-      </c>
-      <c r="B101" t="s">
-        <v>311</v>
       </c>
       <c r="C101">
         <v>557335</v>
@@ -4272,16 +5597,31 @@
       <c r="E101" t="s">
         <v>14</v>
       </c>
-      <c r="F101" t="s">
+      <c r="F101" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="G101" t="s">
+        <v>460</v>
+      </c>
+      <c r="I101" t="s">
+        <v>461</v>
+      </c>
+      <c r="J101" t="s">
+        <v>462</v>
+      </c>
+      <c r="K101" t="s">
+        <v>462</v>
+      </c>
+      <c r="L101" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12">
+      <c r="A102" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
+      <c r="B102" t="s">
         <v>313</v>
-      </c>
-      <c r="B102" t="s">
-        <v>314</v>
       </c>
       <c r="C102">
         <v>562512</v>
@@ -4292,16 +5632,28 @@
       <c r="E102" t="s">
         <v>14</v>
       </c>
-      <c r="F102" t="s">
+      <c r="F102" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="G102" t="s">
+        <v>479</v>
+      </c>
+      <c r="I102" t="s">
+        <v>458</v>
+      </c>
+      <c r="K102" t="s">
+        <v>462</v>
+      </c>
+      <c r="L102" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12">
+      <c r="A103" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
+      <c r="B103" t="s">
         <v>316</v>
-      </c>
-      <c r="B103" t="s">
-        <v>317</v>
       </c>
       <c r="C103">
         <v>583161</v>
@@ -4312,16 +5664,22 @@
       <c r="E103" t="s">
         <v>14</v>
       </c>
-      <c r="F103" t="s">
+      <c r="F103" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="G103" t="s">
+        <v>485</v>
+      </c>
+      <c r="I103" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12">
+      <c r="A104" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
+      <c r="B104" t="s">
         <v>319</v>
-      </c>
-      <c r="B104" t="s">
-        <v>320</v>
       </c>
       <c r="C104">
         <v>602886</v>
@@ -4332,16 +5690,22 @@
       <c r="E104" t="s">
         <v>14</v>
       </c>
-      <c r="F104" t="s">
+      <c r="F104" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="G104" t="s">
+        <v>478</v>
+      </c>
+      <c r="I104" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12">
+      <c r="A105" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
+      <c r="B105" t="s">
         <v>322</v>
-      </c>
-      <c r="B105" t="s">
-        <v>323</v>
       </c>
       <c r="C105">
         <v>632306</v>
@@ -4352,16 +5716,28 @@
       <c r="E105" t="s">
         <v>14</v>
       </c>
-      <c r="F105" t="s">
+      <c r="F105" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="G105" t="s">
+        <v>464</v>
+      </c>
+      <c r="I105" t="s">
+        <v>458</v>
+      </c>
+      <c r="K105" t="s">
+        <v>462</v>
+      </c>
+      <c r="L105" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12">
+      <c r="A106" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" t="s">
+      <c r="B106" t="s">
         <v>325</v>
-      </c>
-      <c r="B106" t="s">
-        <v>326</v>
       </c>
       <c r="C106">
         <v>645246</v>
@@ -4372,16 +5748,22 @@
       <c r="E106" t="s">
         <v>14</v>
       </c>
-      <c r="F106" t="s">
+      <c r="F106" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="G106" t="s">
+        <v>459</v>
+      </c>
+      <c r="I106" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12">
+      <c r="A107" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
+      <c r="B107" t="s">
         <v>328</v>
-      </c>
-      <c r="B107" t="s">
-        <v>329</v>
       </c>
       <c r="C107">
         <v>656977</v>
@@ -4392,16 +5774,25 @@
       <c r="E107" t="s">
         <v>14</v>
       </c>
-      <c r="F107" t="s">
+      <c r="F107" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="G107" t="s">
+        <v>459</v>
+      </c>
+      <c r="I107" t="s">
+        <v>458</v>
+      </c>
+      <c r="L107" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12">
+      <c r="A108" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" t="s">
+      <c r="B108" t="s">
         <v>331</v>
-      </c>
-      <c r="B108" t="s">
-        <v>332</v>
       </c>
       <c r="C108">
         <v>661923</v>
@@ -4412,16 +5803,25 @@
       <c r="E108" t="s">
         <v>14</v>
       </c>
-      <c r="F108" t="s">
+      <c r="F108" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="G108" t="s">
+        <v>457</v>
+      </c>
+      <c r="I108" t="s">
+        <v>458</v>
+      </c>
+      <c r="L108" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12">
+      <c r="A109" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" t="s">
+      <c r="B109" t="s">
         <v>334</v>
-      </c>
-      <c r="B109" t="s">
-        <v>335</v>
       </c>
       <c r="C109">
         <v>697114</v>
@@ -4432,16 +5832,31 @@
       <c r="E109" t="s">
         <v>14</v>
       </c>
-      <c r="F109" t="s">
+      <c r="F109" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="G109" t="s">
+        <v>459</v>
+      </c>
+      <c r="I109" t="s">
+        <v>461</v>
+      </c>
+      <c r="J109" t="s">
+        <v>462</v>
+      </c>
+      <c r="K109" t="s">
+        <v>462</v>
+      </c>
+      <c r="L109" s="4" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12">
+      <c r="A110" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" t="s">
+      <c r="B110" t="s">
         <v>337</v>
-      </c>
-      <c r="B110" t="s">
-        <v>338</v>
       </c>
       <c r="C110">
         <v>727003</v>
@@ -4452,16 +5867,28 @@
       <c r="E110" t="s">
         <v>14</v>
       </c>
-      <c r="F110" t="s">
+      <c r="F110" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="G110" t="s">
+        <v>460</v>
+      </c>
+      <c r="I110" t="s">
+        <v>458</v>
+      </c>
+      <c r="K110" t="s">
+        <v>462</v>
+      </c>
+      <c r="L110" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12">
+      <c r="A111" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" t="s">
+      <c r="B111" t="s">
         <v>340</v>
-      </c>
-      <c r="B111" t="s">
-        <v>341</v>
       </c>
       <c r="C111">
         <v>732292</v>
@@ -4472,16 +5899,28 @@
       <c r="E111" t="s">
         <v>14</v>
       </c>
-      <c r="F111" t="s">
+      <c r="F111" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="G111" t="s">
+        <v>479</v>
+      </c>
+      <c r="I111" t="s">
+        <v>458</v>
+      </c>
+      <c r="K111" t="s">
+        <v>462</v>
+      </c>
+      <c r="L111" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12">
+      <c r="A112" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" t="s">
+      <c r="B112" t="s">
         <v>343</v>
-      </c>
-      <c r="B112" t="s">
-        <v>344</v>
       </c>
       <c r="C112">
         <v>769333</v>
@@ -4492,16 +5931,22 @@
       <c r="E112" t="s">
         <v>14</v>
       </c>
-      <c r="F112" t="s">
+      <c r="F112" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="G112" t="s">
+        <v>459</v>
+      </c>
+      <c r="I112" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12">
+      <c r="A113" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" t="s">
+      <c r="B113" t="s">
         <v>346</v>
-      </c>
-      <c r="B113" t="s">
-        <v>347</v>
       </c>
       <c r="C113">
         <v>771435</v>
@@ -4512,16 +5957,31 @@
       <c r="E113" t="s">
         <v>14</v>
       </c>
-      <c r="F113" t="s">
+      <c r="F113" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="G113" t="s">
+        <v>468</v>
+      </c>
+      <c r="I113" t="s">
+        <v>461</v>
+      </c>
+      <c r="J113" t="s">
+        <v>462</v>
+      </c>
+      <c r="K113" t="s">
+        <v>462</v>
+      </c>
+      <c r="L113" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12">
+      <c r="A114" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A114" t="s">
+      <c r="B114" t="s">
         <v>349</v>
-      </c>
-      <c r="B114" t="s">
-        <v>350</v>
       </c>
       <c r="C114">
         <v>773916</v>
@@ -4532,16 +5992,31 @@
       <c r="E114" t="s">
         <v>14</v>
       </c>
-      <c r="F114" t="s">
+      <c r="F114" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="G114" t="s">
+        <v>464</v>
+      </c>
+      <c r="I114" t="s">
+        <v>461</v>
+      </c>
+      <c r="J114" t="s">
+        <v>462</v>
+      </c>
+      <c r="K114" t="s">
+        <v>462</v>
+      </c>
+      <c r="L114" s="4" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12">
+      <c r="A115" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" t="s">
+      <c r="B115" t="s">
         <v>352</v>
-      </c>
-      <c r="B115" t="s">
-        <v>353</v>
       </c>
       <c r="C115">
         <v>783533</v>
@@ -4552,16 +6027,28 @@
       <c r="E115" t="s">
         <v>14</v>
       </c>
-      <c r="F115" t="s">
+      <c r="F115" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="G115" t="s">
+        <v>485</v>
+      </c>
+      <c r="I115" t="s">
+        <v>461</v>
+      </c>
+      <c r="K115" t="s">
+        <v>462</v>
+      </c>
+      <c r="L115" s="4" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12">
+      <c r="A116" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
+      <c r="B116" t="s">
         <v>355</v>
-      </c>
-      <c r="B116" t="s">
-        <v>356</v>
       </c>
       <c r="C116">
         <v>790828</v>
@@ -4572,16 +6059,22 @@
       <c r="E116" t="s">
         <v>14</v>
       </c>
-      <c r="F116" t="s">
+      <c r="F116" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="G116" t="s">
+        <v>457</v>
+      </c>
+      <c r="I116" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12">
+      <c r="A117" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
+      <c r="B117" t="s">
         <v>358</v>
-      </c>
-      <c r="B117" t="s">
-        <v>359</v>
       </c>
       <c r="C117">
         <v>805729</v>
@@ -4592,16 +6085,22 @@
       <c r="E117" t="s">
         <v>14</v>
       </c>
-      <c r="F117" t="s">
+      <c r="F117" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="G117" t="s">
+        <v>468</v>
+      </c>
+      <c r="I117" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12">
+      <c r="A118" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
+      <c r="B118" t="s">
         <v>361</v>
-      </c>
-      <c r="B118" t="s">
-        <v>362</v>
       </c>
       <c r="C118">
         <v>854899</v>
@@ -4612,16 +6111,31 @@
       <c r="E118" t="s">
         <v>14</v>
       </c>
-      <c r="F118" t="s">
+      <c r="F118" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="G118" t="s">
+        <v>460</v>
+      </c>
+      <c r="I118" t="s">
+        <v>461</v>
+      </c>
+      <c r="J118" t="s">
+        <v>462</v>
+      </c>
+      <c r="K118" t="s">
+        <v>462</v>
+      </c>
+      <c r="L118" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12">
+      <c r="A119" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
+      <c r="B119" t="s">
         <v>364</v>
-      </c>
-      <c r="B119" t="s">
-        <v>365</v>
       </c>
       <c r="C119">
         <v>862333</v>
@@ -4632,16 +6146,22 @@
       <c r="E119" t="s">
         <v>14</v>
       </c>
-      <c r="F119" t="s">
+      <c r="F119" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="G119" t="s">
+        <v>486</v>
+      </c>
+      <c r="I119" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12">
+      <c r="A120" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" t="s">
+      <c r="B120" t="s">
         <v>367</v>
-      </c>
-      <c r="B120" t="s">
-        <v>368</v>
       </c>
       <c r="C120">
         <v>870563</v>
@@ -4652,16 +6172,22 @@
       <c r="E120" t="s">
         <v>14</v>
       </c>
-      <c r="F120" t="s">
+      <c r="F120" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="G120" t="s">
+        <v>464</v>
+      </c>
+      <c r="I120" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12">
+      <c r="A121" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" t="s">
+      <c r="B121" t="s">
         <v>370</v>
-      </c>
-      <c r="B121" t="s">
-        <v>371</v>
       </c>
       <c r="C121">
         <v>941292</v>
@@ -4672,16 +6198,22 @@
       <c r="E121" t="s">
         <v>14</v>
       </c>
-      <c r="F121" t="s">
+      <c r="F121" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="G121" t="s">
+        <v>459</v>
+      </c>
+      <c r="I121" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12">
+      <c r="A122" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" t="s">
+      <c r="B122" t="s">
         <v>373</v>
-      </c>
-      <c r="B122" t="s">
-        <v>374</v>
       </c>
       <c r="C122">
         <v>1186693</v>
@@ -4690,18 +6222,27 @@
         <v>43032.973530092589</v>
       </c>
       <c r="E122" t="s">
+        <v>374</v>
+      </c>
+      <c r="F122" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="F122" t="s">
+      <c r="G122" t="s">
+        <v>478</v>
+      </c>
+      <c r="I122" t="s">
+        <v>458</v>
+      </c>
+      <c r="K122" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12">
+      <c r="A123" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A123" t="s">
+      <c r="B123" t="s">
         <v>377</v>
-      </c>
-      <c r="B123" t="s">
-        <v>378</v>
       </c>
       <c r="C123">
         <v>1253419</v>
@@ -4710,18 +6251,36 @@
         <v>43034.247835648152</v>
       </c>
       <c r="E123" t="s">
-        <v>375</v>
-      </c>
-      <c r="F123" t="s">
+        <v>374</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="G123" t="s">
+        <v>486</v>
+      </c>
+      <c r="H123" t="s">
+        <v>464</v>
+      </c>
+      <c r="I123" t="s">
+        <v>461</v>
+      </c>
+      <c r="J123" t="s">
+        <v>462</v>
+      </c>
+      <c r="K123" t="s">
+        <v>462</v>
+      </c>
+      <c r="L123" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12">
+      <c r="A124" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" t="s">
+      <c r="B124" t="s">
         <v>380</v>
-      </c>
-      <c r="B124" t="s">
-        <v>381</v>
       </c>
       <c r="C124">
         <v>1278292</v>
@@ -4730,18 +6289,30 @@
         <v>43034.675138888888</v>
       </c>
       <c r="E124" t="s">
-        <v>375</v>
-      </c>
-      <c r="F124" t="s">
+        <v>374</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="G124" t="s">
+        <v>479</v>
+      </c>
+      <c r="I124" t="s">
+        <v>461</v>
+      </c>
+      <c r="K124" t="s">
+        <v>462</v>
+      </c>
+      <c r="L124" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12">
+      <c r="A125" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A125" t="s">
+      <c r="B125" t="s">
         <v>383</v>
-      </c>
-      <c r="B125" t="s">
-        <v>384</v>
       </c>
       <c r="C125">
         <v>1309521</v>
@@ -4750,18 +6321,24 @@
         <v>43064.861226851855</v>
       </c>
       <c r="E125" t="s">
-        <v>375</v>
-      </c>
-      <c r="F125" t="s">
+        <v>374</v>
+      </c>
+      <c r="F125" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="G125" t="s">
+        <v>464</v>
+      </c>
+      <c r="I125" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12">
+      <c r="A126" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" t="s">
+      <c r="B126" t="s">
         <v>386</v>
-      </c>
-      <c r="B126" t="s">
-        <v>387</v>
       </c>
       <c r="C126">
         <v>1382254</v>
@@ -4770,18 +6347,36 @@
         <v>43036.264166666668</v>
       </c>
       <c r="E126" t="s">
-        <v>375</v>
-      </c>
-      <c r="F126" t="s">
+        <v>374</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="G126" t="s">
+        <v>459</v>
+      </c>
+      <c r="H126" t="s">
+        <v>485</v>
+      </c>
+      <c r="I126" t="s">
+        <v>458</v>
+      </c>
+      <c r="J126" t="s">
+        <v>462</v>
+      </c>
+      <c r="K126" t="s">
+        <v>462</v>
+      </c>
+      <c r="L126" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12">
+      <c r="A127" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" t="s">
+      <c r="B127" t="s">
         <v>389</v>
-      </c>
-      <c r="B127" t="s">
-        <v>390</v>
       </c>
       <c r="C127">
         <v>1407676</v>
@@ -4790,18 +6385,24 @@
         <v>43040.927222222221</v>
       </c>
       <c r="E127" t="s">
-        <v>375</v>
-      </c>
-      <c r="F127" t="s">
+        <v>374</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="G127" t="s">
+        <v>457</v>
+      </c>
+      <c r="I127" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12">
+      <c r="A128" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" t="s">
+      <c r="B128" t="s">
         <v>392</v>
-      </c>
-      <c r="B128" t="s">
-        <v>393</v>
       </c>
       <c r="C128">
         <v>1670374</v>
@@ -4810,18 +6411,27 @@
         <v>43045.513726851852</v>
       </c>
       <c r="E128" t="s">
-        <v>375</v>
-      </c>
-      <c r="F128" t="s">
+        <v>374</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="G128" t="s">
+        <v>478</v>
+      </c>
+      <c r="I128" t="s">
+        <v>458</v>
+      </c>
+      <c r="L128" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12">
+      <c r="A129" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" t="s">
+      <c r="B129" t="s">
         <v>395</v>
-      </c>
-      <c r="B129" t="s">
-        <v>396</v>
       </c>
       <c r="C129">
         <v>1740133</v>
@@ -4830,18 +6440,27 @@
         <v>43046.696701388886</v>
       </c>
       <c r="E129" t="s">
-        <v>375</v>
-      </c>
-      <c r="F129" t="s">
+        <v>374</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="G129" t="s">
+        <v>548</v>
+      </c>
+      <c r="I129" t="s">
+        <v>458</v>
+      </c>
+      <c r="K129" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12">
+      <c r="A130" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" t="s">
+      <c r="B130" t="s">
         <v>398</v>
-      </c>
-      <c r="B130" t="s">
-        <v>399</v>
       </c>
       <c r="C130">
         <v>1749903</v>
@@ -4850,18 +6469,33 @@
         <v>43046.735185185185</v>
       </c>
       <c r="E130" t="s">
-        <v>375</v>
-      </c>
-      <c r="F130" t="s">
+        <v>374</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="G130" t="s">
+        <v>485</v>
+      </c>
+      <c r="I130" t="s">
+        <v>461</v>
+      </c>
+      <c r="J130" t="s">
+        <v>462</v>
+      </c>
+      <c r="K130" t="s">
+        <v>462</v>
+      </c>
+      <c r="L130" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12">
+      <c r="A131" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" t="s">
+      <c r="B131" t="s">
         <v>401</v>
-      </c>
-      <c r="B131" t="s">
-        <v>402</v>
       </c>
       <c r="C131">
         <v>1803445</v>
@@ -4870,18 +6504,27 @@
         <v>43026.062002314815</v>
       </c>
       <c r="E131" t="s">
-        <v>375</v>
-      </c>
-      <c r="F131" t="s">
+        <v>374</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="G131" t="s">
+        <v>478</v>
+      </c>
+      <c r="I131" t="s">
+        <v>458</v>
+      </c>
+      <c r="L131" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12">
+      <c r="A132" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" t="s">
+      <c r="B132" t="s">
         <v>404</v>
-      </c>
-      <c r="B132" t="s">
-        <v>405</v>
       </c>
       <c r="C132">
         <v>1839193</v>
@@ -4890,18 +6533,33 @@
         <v>43025.822465277779</v>
       </c>
       <c r="E132" t="s">
-        <v>375</v>
-      </c>
-      <c r="F132" t="s">
+        <v>374</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="G132" t="s">
+        <v>464</v>
+      </c>
+      <c r="I132" t="s">
+        <v>461</v>
+      </c>
+      <c r="J132" t="s">
+        <v>462</v>
+      </c>
+      <c r="K132" t="s">
+        <v>462</v>
+      </c>
+      <c r="L132" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="133" spans="1:12">
+      <c r="A133" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" t="s">
+      <c r="B133" t="s">
         <v>407</v>
-      </c>
-      <c r="B133" t="s">
-        <v>408</v>
       </c>
       <c r="C133">
         <v>2098666</v>
@@ -4910,18 +6568,24 @@
         <v>43059.885428240741</v>
       </c>
       <c r="E133" t="s">
-        <v>375</v>
-      </c>
-      <c r="F133" t="s">
+        <v>374</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="G133" t="s">
+        <v>457</v>
+      </c>
+      <c r="I133" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12">
+      <c r="A134" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" t="s">
+      <c r="B134" t="s">
         <v>410</v>
-      </c>
-      <c r="B134" t="s">
-        <v>411</v>
       </c>
       <c r="C134">
         <v>227792</v>
@@ -4930,18 +6594,24 @@
         <v>43013.326851851853</v>
       </c>
       <c r="E134" t="s">
-        <v>375</v>
-      </c>
-      <c r="F134" t="s">
+        <v>374</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="G134" t="s">
+        <v>466</v>
+      </c>
+      <c r="I134" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12">
+      <c r="A135" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" t="s">
+      <c r="B135" t="s">
         <v>413</v>
-      </c>
-      <c r="B135" t="s">
-        <v>414</v>
       </c>
       <c r="C135">
         <v>2319161</v>
@@ -4950,18 +6620,36 @@
         <v>43052.498333333337</v>
       </c>
       <c r="E135" t="s">
-        <v>375</v>
-      </c>
-      <c r="F135" t="s">
+        <v>374</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="G135" t="s">
+        <v>478</v>
+      </c>
+      <c r="H135" t="s">
+        <v>485</v>
+      </c>
+      <c r="I135" t="s">
+        <v>461</v>
+      </c>
+      <c r="J135" t="s">
+        <v>462</v>
+      </c>
+      <c r="K135" t="s">
+        <v>462</v>
+      </c>
+      <c r="L135" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12">
+      <c r="A136" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" t="s">
+      <c r="B136" t="s">
         <v>416</v>
-      </c>
-      <c r="B136" t="s">
-        <v>417</v>
       </c>
       <c r="C136">
         <v>2578139</v>
@@ -4970,18 +6658,24 @@
         <v>43065.84097222222</v>
       </c>
       <c r="E136" t="s">
-        <v>375</v>
-      </c>
-      <c r="F136" t="s">
+        <v>374</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="G136" t="s">
+        <v>457</v>
+      </c>
+      <c r="I136" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="137" spans="1:12">
+      <c r="A137" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" t="s">
+      <c r="B137" t="s">
         <v>419</v>
-      </c>
-      <c r="B137" t="s">
-        <v>420</v>
       </c>
       <c r="C137">
         <v>2585725</v>
@@ -4990,18 +6684,33 @@
         <v>43055.987650462965</v>
       </c>
       <c r="E137" t="s">
-        <v>375</v>
-      </c>
-      <c r="F137" t="s">
+        <v>374</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="G137" t="s">
+        <v>468</v>
+      </c>
+      <c r="I137" t="s">
+        <v>461</v>
+      </c>
+      <c r="J137" t="s">
+        <v>462</v>
+      </c>
+      <c r="K137" t="s">
+        <v>462</v>
+      </c>
+      <c r="L137" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="138" spans="1:12">
+      <c r="A138" t="s">
         <v>421</v>
       </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A138" t="s">
+      <c r="B138" t="s">
         <v>422</v>
-      </c>
-      <c r="B138" t="s">
-        <v>423</v>
       </c>
       <c r="C138">
         <v>2706125</v>
@@ -5010,18 +6719,24 @@
         <v>43058.935428240744</v>
       </c>
       <c r="E138" t="s">
-        <v>375</v>
-      </c>
-      <c r="F138" t="s">
+        <v>374</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="G138" t="s">
+        <v>472</v>
+      </c>
+      <c r="I138" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12">
+      <c r="A139" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" t="s">
+      <c r="B139" t="s">
         <v>425</v>
-      </c>
-      <c r="B139" t="s">
-        <v>426</v>
       </c>
       <c r="C139">
         <v>2783714</v>
@@ -5030,18 +6745,24 @@
         <v>43060.723194444443</v>
       </c>
       <c r="E139" t="s">
-        <v>375</v>
-      </c>
-      <c r="F139" t="s">
+        <v>374</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="G139" t="s">
+        <v>478</v>
+      </c>
+      <c r="I139" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="140" spans="1:12">
+      <c r="A140" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" t="s">
+      <c r="B140" t="s">
         <v>428</v>
-      </c>
-      <c r="B140" t="s">
-        <v>429</v>
       </c>
       <c r="C140">
         <v>2814109</v>
@@ -5050,18 +6771,36 @@
         <v>43066.090682870374</v>
       </c>
       <c r="E140" t="s">
-        <v>375</v>
-      </c>
-      <c r="F140" t="s">
+        <v>374</v>
+      </c>
+      <c r="F140" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="G140" t="s">
+        <v>551</v>
+      </c>
+      <c r="H140" t="s">
+        <v>472</v>
+      </c>
+      <c r="I140" t="s">
+        <v>461</v>
+      </c>
+      <c r="J140" t="s">
+        <v>462</v>
+      </c>
+      <c r="K140" t="s">
+        <v>462</v>
+      </c>
+      <c r="L140" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="141" spans="1:12">
+      <c r="A141" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A141" t="s">
+      <c r="B141" t="s">
         <v>431</v>
-      </c>
-      <c r="B141" t="s">
-        <v>432</v>
       </c>
       <c r="C141">
         <v>2925107</v>
@@ -5070,18 +6809,36 @@
         <v>43068.131597222222</v>
       </c>
       <c r="E141" t="s">
-        <v>375</v>
-      </c>
-      <c r="F141" t="s">
+        <v>374</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="G141" t="s">
+        <v>485</v>
+      </c>
+      <c r="H141" t="s">
+        <v>468</v>
+      </c>
+      <c r="I141" t="s">
+        <v>461</v>
+      </c>
+      <c r="J141" t="s">
+        <v>462</v>
+      </c>
+      <c r="K141" t="s">
+        <v>462</v>
+      </c>
+      <c r="L141" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12">
+      <c r="A142" t="s">
         <v>433</v>
       </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" t="s">
+      <c r="B142" t="s">
         <v>434</v>
-      </c>
-      <c r="B142" t="s">
-        <v>435</v>
       </c>
       <c r="C142">
         <v>441977</v>
@@ -5090,18 +6847,33 @@
         <v>43019.448148148149</v>
       </c>
       <c r="E142" t="s">
-        <v>375</v>
-      </c>
-      <c r="F142" t="s">
+        <v>374</v>
+      </c>
+      <c r="F142" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="G142" t="s">
+        <v>479</v>
+      </c>
+      <c r="I142" t="s">
+        <v>461</v>
+      </c>
+      <c r="J142" t="s">
+        <v>462</v>
+      </c>
+      <c r="K142" t="s">
+        <v>462</v>
+      </c>
+      <c r="L142" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12">
+      <c r="A143" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" t="s">
+      <c r="B143" t="s">
         <v>437</v>
-      </c>
-      <c r="B143" t="s">
-        <v>438</v>
       </c>
       <c r="C143">
         <v>466955</v>
@@ -5110,18 +6882,36 @@
         <v>43070.183796296296</v>
       </c>
       <c r="E143" t="s">
-        <v>375</v>
-      </c>
-      <c r="F143" t="s">
+        <v>374</v>
+      </c>
+      <c r="F143" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="G143" t="s">
+        <v>464</v>
+      </c>
+      <c r="H143" t="s">
+        <v>459</v>
+      </c>
+      <c r="I143" t="s">
+        <v>461</v>
+      </c>
+      <c r="J143" t="s">
+        <v>462</v>
+      </c>
+      <c r="K143" t="s">
+        <v>462</v>
+      </c>
+      <c r="L143" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12">
+      <c r="A144" t="s">
         <v>439</v>
       </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" t="s">
+      <c r="B144" t="s">
         <v>440</v>
-      </c>
-      <c r="B144" t="s">
-        <v>441</v>
       </c>
       <c r="C144">
         <v>596428</v>
@@ -5130,18 +6920,27 @@
         <v>43072.797789351855</v>
       </c>
       <c r="E144" t="s">
-        <v>375</v>
-      </c>
-      <c r="F144" t="s">
+        <v>374</v>
+      </c>
+      <c r="F144" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="G144" t="s">
+        <v>457</v>
+      </c>
+      <c r="I144" t="s">
+        <v>458</v>
+      </c>
+      <c r="K144" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9">
+      <c r="A145" t="s">
         <v>442</v>
       </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A145" t="s">
+      <c r="B145" t="s">
         <v>443</v>
-      </c>
-      <c r="B145" t="s">
-        <v>444</v>
       </c>
       <c r="C145">
         <v>607619</v>
@@ -5150,18 +6949,24 @@
         <v>43061.481365740743</v>
       </c>
       <c r="E145" t="s">
-        <v>375</v>
-      </c>
-      <c r="F145" t="s">
+        <v>374</v>
+      </c>
+      <c r="F145" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="G145" t="s">
+        <v>457</v>
+      </c>
+      <c r="I145" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9">
+      <c r="A146" t="s">
         <v>445</v>
       </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A146" t="s">
+      <c r="B146" t="s">
         <v>446</v>
-      </c>
-      <c r="B146" t="s">
-        <v>447</v>
       </c>
       <c r="C146">
         <v>834249</v>
@@ -5170,18 +6975,24 @@
         <v>43021.311574074076</v>
       </c>
       <c r="E146" t="s">
-        <v>375</v>
-      </c>
-      <c r="F146" t="s">
+        <v>374</v>
+      </c>
+      <c r="F146" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="G146" t="s">
+        <v>478</v>
+      </c>
+      <c r="I146" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9">
+      <c r="A147" t="s">
         <v>448</v>
       </c>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A147" t="s">
+      <c r="B147" t="s">
         <v>449</v>
-      </c>
-      <c r="B147" t="s">
-        <v>450</v>
       </c>
       <c r="C147">
         <v>939713</v>
@@ -5190,18 +7001,24 @@
         <v>43029.774351851855</v>
       </c>
       <c r="E147" t="s">
-        <v>375</v>
-      </c>
-      <c r="F147" t="s">
+        <v>374</v>
+      </c>
+      <c r="F147" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="G147" t="s">
+        <v>481</v>
+      </c>
+      <c r="I147" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9">
+      <c r="A148" t="s">
         <v>451</v>
       </c>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A148" t="s">
+      <c r="B148" t="s">
         <v>452</v>
-      </c>
-      <c r="B148" t="s">
-        <v>453</v>
       </c>
       <c r="C148">
         <v>939721</v>
@@ -5210,18 +7027,24 @@
         <v>43029.769895833335</v>
       </c>
       <c r="E148" t="s">
-        <v>375</v>
-      </c>
-      <c r="F148" t="s">
+        <v>374</v>
+      </c>
+      <c r="F148" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="G148" t="s">
+        <v>457</v>
+      </c>
+      <c r="I148" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9">
+      <c r="A149" t="s">
         <v>454</v>
       </c>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A149" t="s">
+      <c r="B149" t="s">
         <v>455</v>
-      </c>
-      <c r="B149" t="s">
-        <v>456</v>
       </c>
       <c r="C149">
         <v>945991</v>
@@ -5230,10 +7053,16 @@
         <v>43064.694189814814</v>
       </c>
       <c r="E149" t="s">
-        <v>375</v>
-      </c>
-      <c r="F149" t="s">
+        <v>374</v>
+      </c>
+      <c r="F149" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="G149" t="s">
         <v>457</v>
+      </c>
+      <c r="I149" t="s">
+        <v>458</v>
       </c>
     </row>
   </sheetData>

</xml_diff>